<commit_message>
Identify legacy simulator codes explicitly in research map evidence
</commit_message>
<xml_diff>
--- a/outputs/starter-destinations-20261029/starter-destination-catalogue.xlsx
+++ b/outputs/starter-destinations-20261029/starter-destination-catalogue.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Career shortlists" sheetId="1" r:id="R8111e8d3b55540bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogue" sheetId="2" r:id="Rd39747d72c7746ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring" sheetId="3" r:id="Rb265731df7a8498c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aircraft and method" sheetId="4" r:id="R1665cb52825649ac"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custom opportunities" sheetId="5" r:id="R5b9d724ac0374b91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Career shortlists" sheetId="1" r:id="Rd50f0c8e536747bd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogue" sheetId="2" r:id="R8b6d65f62ccf44b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scoring" sheetId="3" r:id="Rd9ba7b63326649d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aircraft and method" sheetId="4" r:id="R1fdc6aec36a74119"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Custom opportunities" sheetId="5" r:id="Rb33a22496ae940c2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2909,7 +2909,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R6" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.1 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYOP returned in 2026-10-27 cache; offset 0.1 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S6" s="15" t="n">
         <x:v>328</x:v>
@@ -3201,7 +3201,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R8" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYEF returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S8" s="15" t="n">
         <x:v>399.7</x:v>
@@ -3347,7 +3347,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R9" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 588.6 NM from real-world point. WRONG-LOCATION ASSOCIATION; hold.</x:v>
+        <x:v>FYKW returned in 2026-10-27 cache; offset 588.6 NM from real-world point. WRONG-LOCATION ASSOCIATION; hold.</x:v>
       </x:c>
       <x:c r="S9" s="15" t="n">
         <x:v>377</x:v>
@@ -3640,7 +3640,7 @@
         <x:v>No aircraft approved by this research. Known paved runway: candidate for fleet-specific AFM/weight/density-altitude assessment.</x:v>
       </x:c>
       <x:c r="R11" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.4 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYRC returned in 2026-10-27 cache; offset 0.4 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S11" s="15" t="n">
         <x:v>346.7</x:v>
@@ -3786,7 +3786,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R12" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.2 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYTK returned in 2026-10-27 cache; offset 0.2 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S12" s="15" t="n">
         <x:v>261.9</x:v>
@@ -3938,7 +3938,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R13" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYOE returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S13" s="15" t="n">
         <x:v>397.7</x:v>
@@ -4082,7 +4082,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R14" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYNP returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S14" s="15" t="n">
         <x:v>300.5</x:v>
@@ -4231,7 +4231,7 @@
         <x:v>No aircraft approved by this research. Known paved runway: candidate for fleet-specific AFM/weight/density-altitude assessment.</x:v>
       </x:c>
       <x:c r="R15" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.1 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYRU returned in 2026-10-27 cache; offset 0.1 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S15" s="15" t="n">
         <x:v>316.2</x:v>
@@ -4382,7 +4382,7 @@
         <x:v>No aircraft approved by this research. Known paved runway: candidate for fleet-specific AFM/weight/density-altitude assessment.</x:v>
       </x:c>
       <x:c r="R16" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYEN returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S16" s="15" t="n">
         <x:v>310.5</x:v>
@@ -4670,7 +4670,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R18" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYOH returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S18" s="15" t="n">
         <x:v>305.2</x:v>
@@ -4817,7 +4817,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R19" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.1 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYKJ returned in 2026-10-27 cache; offset 0.1 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S19" s="15" t="n">
         <x:v>224.2</x:v>
@@ -4963,7 +4963,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R20" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.2 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYOJ returned in 2026-10-27 cache; offset 0.2 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S20" s="15" t="n">
         <x:v>161</x:v>
@@ -5113,7 +5113,7 @@
         <x:v>No aircraft approved by this research. Known paved runway: candidate for fleet-specific AFM/weight/density-altitude assessment.</x:v>
       </x:c>
       <x:c r="R21" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYOS returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S21" s="15" t="n">
         <x:v>298.9</x:v>
@@ -5833,7 +5833,7 @@
         <x:v>No aircraft approved by this research. Known paved runway: candidate for fleet-specific AFM/weight/density-altitude assessment.</x:v>
       </x:c>
       <x:c r="R26" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.4 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYAR returned in 2026-10-27 cache; offset 0.4 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S26" s="15" t="n">
         <x:v>116.8</x:v>
@@ -5984,7 +5984,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R27" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYUS returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S27" s="15" t="n">
         <x:v>148.3</x:v>
@@ -6422,7 +6422,7 @@
         <x:v>No aircraft approved by this research. Known paved runway: candidate for fleet-specific AFM/weight/density-altitude assessment.</x:v>
       </x:c>
       <x:c r="R30" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.3 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYTM returned in 2026-10-27 cache; offset 0.3 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S30" s="15" t="n">
         <x:v>204</x:v>
@@ -6569,7 +6569,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R31" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.3 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYKA returned in 2026-10-27 cache; offset 0.3 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S31" s="15" t="n">
         <x:v>79.6</x:v>
@@ -6716,7 +6716,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R32" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.2 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYSM returned in 2026-10-27 cache; offset 0.2 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S32" s="15" t="n">
         <x:v>139.2</x:v>
@@ -6872,7 +6872,7 @@
         <x:v>No aircraft approved by this research. Known paved runway: candidate for fleet-specific AFM/weight/density-altitude assessment.</x:v>
       </x:c>
       <x:c r="R33" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.1 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYWB returned in 2026-10-27 cache; offset 0.1 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S33" s="15" t="n">
         <x:v>136.5</x:v>
@@ -7168,7 +7168,7 @@
         <x:v>No aircraft approved by this research. Known paved runway: candidate for fleet-specific AFM/weight/density-altitude assessment.</x:v>
       </x:c>
       <x:c r="R35" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYOG returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S35" s="15" t="n">
         <x:v>360.7</x:v>
@@ -7326,7 +7326,7 @@
         <x:v>No aircraft approved by this research. Known paved runway: candidate for fleet-specific AFM/weight/density-altitude assessment.</x:v>
       </x:c>
       <x:c r="R36" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.2 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYLZ returned in 2026-10-27 cache; offset 0.2 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S36" s="15" t="n">
         <x:v>264.8</x:v>
@@ -7480,7 +7480,7 @@
         <x:v>No aircraft approved by this research. Known paved runway: candidate for fleet-specific AFM/weight/density-altitude assessment.</x:v>
       </x:c>
       <x:c r="R37" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.6 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYGF returned in 2026-10-27 cache; offset 0.6 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S37" s="15" t="n">
         <x:v>189.5</x:v>
@@ -7625,7 +7625,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R38" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 317.6 NM from real-world point. WRONG-LOCATION ASSOCIATION; hold.</x:v>
+        <x:v>FYNG returned in 2026-10-27 cache; offset 317.6 NM from real-world point. WRONG-LOCATION ASSOCIATION; hold.</x:v>
       </x:c>
       <x:c r="S38" s="15" t="n">
         <x:v>207.3</x:v>
@@ -7771,7 +7771,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R39" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.4 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYMO returned in 2026-10-27 cache; offset 0.4 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S39" s="15" t="n">
         <x:v>227.7</x:v>
@@ -8211,7 +8211,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R42" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYGK returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S42" s="15" t="n">
         <x:v>136.8</x:v>
@@ -8629,7 +8629,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R45" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 148.0 NM from real-world point. WRONG-LOCATION ASSOCIATION; hold.</x:v>
+        <x:v>FYAD returned in 2026-10-27 cache; offset 148.0 NM from real-world point. WRONG-LOCATION ASSOCIATION; hold.</x:v>
       </x:c>
       <x:c r="S45" s="15" t="n">
         <x:v>173.6</x:v>
@@ -9067,7 +9067,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R48" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 526.4 NM from real-world point. WRONG-LOCATION ASSOCIATION; hold.</x:v>
+        <x:v>FYHV returned in 2026-10-27 cache; offset 526.4 NM from real-world point. WRONG-LOCATION ASSOCIATION; hold.</x:v>
       </x:c>
       <x:c r="S48" s="15" t="n">
         <x:v>415.4</x:v>
@@ -9214,7 +9214,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R49" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 381.5 NM from real-world point. WRONG-LOCATION ASSOCIATION; hold.</x:v>
+        <x:v>FYHO returned in 2026-10-27 cache; offset 381.5 NM from real-world point. WRONG-LOCATION ASSOCIATION; hold.</x:v>
       </x:c>
       <x:c r="S49" s="15" t="n">
         <x:v>293.7</x:v>
@@ -9650,7 +9650,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R52" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.1 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYOO returned in 2026-10-27 cache; offset 0.1 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S52" s="15" t="n">
         <x:v>217.6</x:v>
@@ -9796,7 +9796,7 @@
         <x:v>No aircraft approved by this research. Unknown/conflicting field data: hold performance clearance; assess each type separately.</x:v>
       </x:c>
       <x:c r="R53" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.1 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYME returned in 2026-10-27 cache; offset 0.1 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S53" s="15" t="n">
         <x:v>101.2</x:v>
@@ -11067,7 +11067,7 @@
         <x:v>No aircraft approved by this research. Known paved runway: candidate for fleet-specific AFM/weight/density-altitude assessment.</x:v>
       </x:c>
       <x:c r="R62" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.2 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYWE returned in 2026-10-27 cache; offset 0.2 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S62" s="15" t="n">
         <x:v>0</x:v>
@@ -11211,7 +11211,7 @@
         <x:v>No aircraft approved by this research. Known paved runway: candidate for fleet-specific AFM/weight/density-altitude assessment.</x:v>
       </x:c>
       <x:c r="R63" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYWH returned in 2026-10-27 cache; offset 0.0 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S63" s="15" t="n">
         <x:v>23</x:v>
@@ -11359,7 +11359,7 @@
         <x:v>No aircraft approved by this research. Known paved runway: candidate for fleet-specific AFM/weight/density-altitude assessment.</x:v>
       </x:c>
       <x:c r="R64" s="7" t="str">
-        <x:v>Identifier returned in 2026-10-27 cache; offset 0.1 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
+        <x:v>FYKT returned in 2026-10-27 cache; offset 0.1 NM from real-world point. Database presence only; scenery/runway uninspected.</x:v>
       </x:c>
       <x:c r="S64" s="15" t="n">
         <x:v>242.9</x:v>
@@ -12391,7 +12391,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5e3cc1236ff54c6d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4eccc1586eea42ff"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20016,7 +20016,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7922acddb4664029"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4b69eb9b2d174ccd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -20916,7 +20916,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfaa2a451bd364875"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra1eaea7bd18542d8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>